<commit_message>
Revising test documentation format
</commit_message>
<xml_diff>
--- a/Periplus-Cart-Test-Michael-Ignasius.xlsx
+++ b/Periplus-Cart-Test-Michael-Ignasius.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
   <si>
     <t>End To End Test Cases for Periplus Shopping Cart Feature</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>Severity Level</t>
+  </si>
+  <si>
+    <t>Comments</t>
   </si>
   <si>
     <t>SC-P01</t>
@@ -663,7 +666,7 @@
     <col customWidth="1" min="5" max="5" width="32.13"/>
     <col customWidth="1" min="6" max="6" width="18.13"/>
     <col customWidth="1" min="7" max="7" width="12.38"/>
-    <col customWidth="1" min="8" max="8" width="45.88"/>
+    <col customWidth="1" min="8" max="8" width="38.13"/>
     <col customWidth="1" min="9" max="9" width="11.0"/>
     <col customWidth="1" min="10" max="10" width="22.88"/>
   </cols>
@@ -673,7 +676,6 @@
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -682,7 +684,6 @@
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
@@ -691,7 +692,6 @@
       <c r="B3" s="4">
         <v>46170.0</v>
       </c>
-      <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
@@ -753,558 +753,569 @@
       <c r="G7" s="12" t="s">
         <v>10</v>
       </c>
+      <c r="H7" s="12" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
       <c r="F8" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>15</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H8" s="15"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
       <c r="F9" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>15</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H9" s="15"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
       <c r="F10" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>15</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H10" s="15"/>
     </row>
     <row r="11">
       <c r="A11" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="15"/>
       <c r="F11" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H11" s="15"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
       <c r="F12" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H12" s="15"/>
     </row>
     <row r="13">
       <c r="A13" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
       <c r="F13" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H13" s="15"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
       <c r="F14" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H14" s="15"/>
     </row>
     <row r="15">
       <c r="A15" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
       <c r="F15" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>15</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H15" s="15"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D16" s="18"/>
       <c r="E16" s="19"/>
       <c r="F16" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="H16" s="19"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" s="18"/>
       <c r="E17" s="19"/>
       <c r="F17" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H17" s="19"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D18" s="18"/>
       <c r="E18" s="19"/>
       <c r="F18" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H18" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H18" s="19"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D19" s="18"/>
       <c r="E19" s="19"/>
       <c r="F19" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H19" s="19"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D20" s="18"/>
       <c r="E20" s="19"/>
       <c r="F20" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H20" s="19"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D21" s="18"/>
       <c r="E21" s="19"/>
       <c r="F21" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H21" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H21" s="19"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D22" s="18"/>
       <c r="E22" s="19"/>
       <c r="F22" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H22" s="19"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D23" s="18"/>
       <c r="E23" s="19"/>
       <c r="F23" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H23" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H23" s="19"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="18"/>
       <c r="E24" s="19"/>
       <c r="F24" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H24" s="19"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D25" s="18"/>
       <c r="E25" s="19"/>
       <c r="F25" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H25" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H25" s="19"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D26" s="18"/>
       <c r="E26" s="19"/>
       <c r="F26" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H26" s="19"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D27" s="18"/>
       <c r="E27" s="19"/>
       <c r="F27" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H27" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H27" s="19"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D28" s="18"/>
       <c r="E28" s="19"/>
       <c r="F28" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H28" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H28" s="19"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D29" s="18"/>
       <c r="E29" s="19"/>
       <c r="F29" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H29" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H29" s="19"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D30" s="18"/>
       <c r="E30" s="19"/>
       <c r="F30" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H30" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H30" s="19"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D31" s="18"/>
       <c r="E31" s="19"/>
       <c r="F31" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H31" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H31" s="19"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D32" s="18"/>
       <c r="E32" s="19"/>
       <c r="F32" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="H32" s="19"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D33" s="18"/>
       <c r="E33" s="19"/>
       <c r="F33" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H33" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H33" s="19"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B34" s="17"/>
       <c r="C34" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D34" s="18"/>
       <c r="E34" s="19"/>
       <c r="F34" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H34" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H34" s="19"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B35" s="17"/>
       <c r="C35" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D35" s="18"/>
       <c r="E35" s="19"/>
       <c r="F35" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="H35" s="19"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B36" s="17"/>
       <c r="C36" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D36" s="18"/>
       <c r="E36" s="19"/>
       <c r="F36" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="H36" s="19"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B37" s="17"/>
       <c r="C37" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D37" s="18"/>
       <c r="E37" s="19"/>
       <c r="F37" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H37" s="8"/>
+        <v>52</v>
+      </c>
+      <c r="H37" s="19"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B38" s="20"/>
       <c r="C38" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D38" s="18"/>
       <c r="E38" s="19"/>
       <c r="F38" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H38" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="H38" s="19"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="5"/>
@@ -5974,10 +5985,10 @@
   <mergeCells count="6">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:G3"/>
     <mergeCell ref="B8:B38"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G8:G38">

</xml_diff>